<commit_message>
All Order files updated upto 18 aug 2026 Tuesday
</commit_message>
<xml_diff>
--- a/ORDER_MGMT/regular_order_mgmt/order_files/Mapped_Expired_OrderBook_Equity_17aug26_Mon.xlsx
+++ b/ORDER_MGMT/regular_order_mgmt/order_files/Mapped_Expired_OrderBook_Equity_17aug26_Mon.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\python\stocks\ORDER_MGMT\regular_order_mgmt\order_files\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{ADF47EC7-948D-4337-937D-6251E2AD8A7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95C665C0-75E7-4854-9802-4C40C3CB1440}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1193,7 +1193,6 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr filterMode="1"/>
   <dimension ref="A1:K238"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
@@ -1236,7 +1235,7 @@
       </c>
       <c r="K1" s="17"/>
     </row>
-    <row r="2" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="10" t="s">
         <v>85</v>
       </c>
@@ -1267,7 +1266,7 @@
       <c r="J2" s="17"/>
       <c r="K2" s="17"/>
     </row>
-    <row r="3" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A3" s="5">
         <v>46244.767361111109</v>
       </c>
@@ -1298,7 +1297,7 @@
       <c r="J3" s="17"/>
       <c r="K3" s="17"/>
     </row>
-    <row r="4" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="4" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A4" s="10" t="s">
         <v>85</v>
       </c>
@@ -1329,7 +1328,7 @@
       <c r="J4" s="17"/>
       <c r="K4" s="17"/>
     </row>
-    <row r="5" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="5" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A5" s="10" t="s">
         <v>85</v>
       </c>
@@ -1360,7 +1359,7 @@
       <c r="J5" s="17"/>
       <c r="K5" s="17"/>
     </row>
-    <row r="6" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="6" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A6" s="10" t="s">
         <v>85</v>
       </c>
@@ -1391,7 +1390,7 @@
       <c r="J6" s="17"/>
       <c r="K6" s="17"/>
     </row>
-    <row r="7" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="7" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A7" s="10" t="s">
         <v>85</v>
       </c>
@@ -1422,7 +1421,7 @@
       <c r="J7" s="17"/>
       <c r="K7" s="17"/>
     </row>
-    <row r="8" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="8" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="5">
         <v>46241.6875</v>
       </c>
@@ -1453,7 +1452,7 @@
       <c r="J8" s="17"/>
       <c r="K8" s="17"/>
     </row>
-    <row r="9" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="9" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="5">
         <v>46240.6875</v>
       </c>
@@ -1484,7 +1483,7 @@
       <c r="J9" s="17"/>
       <c r="K9" s="17"/>
     </row>
-    <row r="10" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="10" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="5">
         <v>46244.635416666664</v>
       </c>
@@ -1515,7 +1514,7 @@
       <c r="J10" s="17"/>
       <c r="K10" s="17"/>
     </row>
-    <row r="11" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="11" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="10" t="s">
         <v>85</v>
       </c>
@@ -1546,7 +1545,7 @@
       <c r="J11" s="17"/>
       <c r="K11" s="17"/>
     </row>
-    <row r="12" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="12" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="5">
         <v>46150.635416666664</v>
       </c>
@@ -1577,7 +1576,7 @@
       <c r="J12" s="17"/>
       <c r="K12" s="17"/>
     </row>
-    <row r="13" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="13" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="5">
         <v>46150.789583333331</v>
       </c>
@@ -1608,7 +1607,7 @@
       <c r="J13" s="17"/>
       <c r="K13" s="17"/>
     </row>
-    <row r="14" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="14" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="5">
         <v>46248.770833333336</v>
       </c>
@@ -1639,7 +1638,7 @@
       <c r="J14" s="17"/>
       <c r="K14" s="17"/>
     </row>
-    <row r="15" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="15" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="5">
         <v>46181.6875</v>
       </c>
@@ -1670,7 +1669,7 @@
       <c r="J15" s="17"/>
       <c r="K15" s="17"/>
     </row>
-    <row r="16" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="16" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="5">
         <v>46181.635416666664</v>
       </c>
@@ -1701,7 +1700,7 @@
       <c r="J16" s="17"/>
       <c r="K16" s="17"/>
     </row>
-    <row r="17" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="17" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="10" t="s">
         <v>85</v>
       </c>
@@ -1732,7 +1731,7 @@
       <c r="J17" s="17"/>
       <c r="K17" s="17"/>
     </row>
-    <row r="18" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="18" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="5">
         <v>46239.788888888892</v>
       </c>
@@ -1763,7 +1762,7 @@
       <c r="J18" s="17"/>
       <c r="K18" s="17"/>
     </row>
-    <row r="19" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="19" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="5">
         <v>46246.644444444442</v>
       </c>
@@ -1794,7 +1793,7 @@
       <c r="J19" s="17"/>
       <c r="K19" s="17"/>
     </row>
-    <row r="20" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="20" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="5">
         <v>46251.688622685186</v>
       </c>
@@ -1825,7 +1824,7 @@
       <c r="J20" s="17"/>
       <c r="K20" s="17"/>
     </row>
-    <row r="21" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="21" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="5">
         <v>46334.692361111112</v>
       </c>
@@ -1856,7 +1855,7 @@
       <c r="J21" s="17"/>
       <c r="K21" s="17"/>
     </row>
-    <row r="22" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="22" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="10" t="s">
         <v>85</v>
       </c>
@@ -1887,7 +1886,7 @@
       <c r="J22" s="17"/>
       <c r="K22" s="17"/>
     </row>
-    <row r="23" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="23" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="5">
         <v>46239.635416666664</v>
       </c>
@@ -1918,7 +1917,7 @@
       <c r="J23" s="17"/>
       <c r="K23" s="17"/>
     </row>
-    <row r="24" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="24" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="5">
         <v>46211.635416666664</v>
       </c>
@@ -1949,7 +1948,7 @@
       <c r="J24" s="17"/>
       <c r="K24" s="17"/>
     </row>
-    <row r="25" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="25" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="5">
         <v>46248.768750000003</v>
       </c>
@@ -1980,7 +1979,7 @@
       <c r="J25" s="17"/>
       <c r="K25" s="17"/>
     </row>
-    <row r="26" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="26" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="5">
         <v>46334.635416666664</v>
       </c>
@@ -2011,7 +2010,7 @@
       <c r="J26" s="17"/>
       <c r="K26" s="17"/>
     </row>
-    <row r="27" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="27" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -2042,7 +2041,7 @@
       <c r="J27" s="17"/>
       <c r="K27" s="17"/>
     </row>
-    <row r="28" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="28" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="5">
         <v>46246.689583333333</v>
       </c>
@@ -2073,7 +2072,7 @@
       <c r="J28" s="17"/>
       <c r="K28" s="17"/>
     </row>
-    <row r="29" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="29" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -2104,7 +2103,7 @@
       <c r="J29" s="17"/>
       <c r="K29" s="17"/>
     </row>
-    <row r="30" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="30" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -2137,7 +2136,7 @@
       </c>
       <c r="K30" s="17"/>
     </row>
-    <row r="31" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="31" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="5">
         <v>46245.693055555559</v>
       </c>
@@ -2170,7 +2169,7 @@
       </c>
       <c r="K31" s="17"/>
     </row>
-    <row r="32" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="32" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="5">
         <v>46334.692361111112</v>
       </c>
@@ -2201,7 +2200,7 @@
       <c r="J32" s="17"/>
       <c r="K32" s="17"/>
     </row>
-    <row r="33" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="33" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="5">
         <v>46241.6875</v>
       </c>
@@ -2232,7 +2231,7 @@
       <c r="J33" s="17"/>
       <c r="K33" s="17"/>
     </row>
-    <row r="34" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="34" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="5">
         <v>46240.6875</v>
       </c>
@@ -2263,7 +2262,7 @@
       <c r="J34" s="17"/>
       <c r="K34" s="17"/>
     </row>
-    <row r="35" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="35" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="5">
         <v>46245.693055555559</v>
       </c>
@@ -2294,7 +2293,7 @@
       <c r="J35" s="17"/>
       <c r="K35" s="17"/>
     </row>
-    <row r="36" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="36" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -2327,7 +2326,7 @@
       </c>
       <c r="K36" s="17"/>
     </row>
-    <row r="37" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="37" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -2358,7 +2357,7 @@
       <c r="J37" s="17"/>
       <c r="K37" s="17"/>
     </row>
-    <row r="38" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="38" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="5">
         <v>46245.693055555559</v>
       </c>
@@ -2389,7 +2388,7 @@
       <c r="J38" s="17"/>
       <c r="K38" s="17"/>
     </row>
-    <row r="39" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="39" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="10" t="s">
         <v>85</v>
       </c>
@@ -2420,7 +2419,7 @@
       <c r="J39" s="17"/>
       <c r="K39" s="17"/>
     </row>
-    <row r="40" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="40" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="5">
         <v>46251.688622685186</v>
       </c>
@@ -2451,7 +2450,7 @@
       <c r="J40" s="17"/>
       <c r="K40" s="17"/>
     </row>
-    <row r="41" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="41" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="5">
         <v>46251.635509259257</v>
       </c>
@@ -2482,7 +2481,7 @@
       <c r="J41" s="17"/>
       <c r="K41" s="17"/>
     </row>
-    <row r="42" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="42" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="5">
         <v>46241.6875</v>
       </c>
@@ -2515,7 +2514,7 @@
       </c>
       <c r="K42" s="17"/>
     </row>
-    <row r="43" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="43" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="5">
         <v>46251.688703703701</v>
       </c>
@@ -2548,7 +2547,7 @@
       </c>
       <c r="K43" s="17"/>
     </row>
-    <row r="44" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="44" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="10" t="s">
         <v>85</v>
       </c>
@@ -2579,7 +2578,7 @@
       <c r="J44" s="17"/>
       <c r="K44" s="17"/>
     </row>
-    <row r="45" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="45" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -2610,7 +2609,7 @@
       <c r="J45" s="17"/>
       <c r="K45" s="17"/>
     </row>
-    <row r="46" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="46" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="5">
         <v>46241.76458333333</v>
       </c>
@@ -2641,7 +2640,7 @@
       <c r="J46" s="17"/>
       <c r="K46" s="17"/>
     </row>
-    <row r="47" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="47" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -2674,7 +2673,7 @@
       </c>
       <c r="K47" s="17"/>
     </row>
-    <row r="48" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="48" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -2705,7 +2704,7 @@
       <c r="J48" s="17"/>
       <c r="K48" s="17"/>
     </row>
-    <row r="49" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="49" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -2736,7 +2735,7 @@
       <c r="J49" s="17"/>
       <c r="K49" s="17"/>
     </row>
-    <row r="50" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="50" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="5">
         <v>46364.635416666664</v>
       </c>
@@ -2767,7 +2766,7 @@
       <c r="J50" s="17"/>
       <c r="K50" s="17"/>
     </row>
-    <row r="51" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="51" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -2800,7 +2799,7 @@
       </c>
       <c r="K51" s="17"/>
     </row>
-    <row r="52" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="52" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="5">
         <v>46251.688634259262</v>
       </c>
@@ -2833,7 +2832,7 @@
       </c>
       <c r="K52" s="17"/>
     </row>
-    <row r="53" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="53" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -2864,7 +2863,7 @@
       <c r="J53" s="17"/>
       <c r="K53" s="17"/>
     </row>
-    <row r="54" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="54" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="5">
         <v>46334.692361111112</v>
       </c>
@@ -2895,7 +2894,7 @@
       <c r="J54" s="17"/>
       <c r="K54" s="17"/>
     </row>
-    <row r="55" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="55" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -2926,7 +2925,7 @@
       <c r="J55" s="17"/>
       <c r="K55" s="17"/>
     </row>
-    <row r="56" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="56" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -2959,7 +2958,7 @@
       </c>
       <c r="K56" s="17"/>
     </row>
-    <row r="57" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="57" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="5">
         <v>46251.688715277778</v>
       </c>
@@ -2992,7 +2991,7 @@
       </c>
       <c r="K57" s="17"/>
     </row>
-    <row r="58" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="58" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -3023,7 +3022,7 @@
       <c r="J58" s="17"/>
       <c r="K58" s="17"/>
     </row>
-    <row r="59" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="59" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="10" t="s">
         <v>85</v>
       </c>
@@ -3054,7 +3053,7 @@
       <c r="J59" s="17"/>
       <c r="K59" s="17"/>
     </row>
-    <row r="60" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="60" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="5">
         <v>46241.765277777777</v>
       </c>
@@ -3085,7 +3084,7 @@
       <c r="J60" s="17"/>
       <c r="K60" s="17"/>
     </row>
-    <row r="61" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="61" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -3118,7 +3117,7 @@
       </c>
       <c r="K61" s="17"/>
     </row>
-    <row r="62" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="62" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -3149,7 +3148,7 @@
       <c r="J62" s="17"/>
       <c r="K62" s="17"/>
     </row>
-    <row r="63" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="63" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="10" t="s">
         <v>85</v>
       </c>
@@ -3180,7 +3179,7 @@
       <c r="J63" s="17"/>
       <c r="K63" s="17"/>
     </row>
-    <row r="64" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="64" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="5">
         <v>46211.6875</v>
       </c>
@@ -3211,7 +3210,7 @@
       <c r="J64" s="17"/>
       <c r="K64" s="17"/>
     </row>
-    <row r="65" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="65" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -3242,7 +3241,7 @@
       <c r="J65" s="17"/>
       <c r="K65" s="17"/>
     </row>
-    <row r="66" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="66" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -3273,7 +3272,7 @@
       <c r="J66" s="17"/>
       <c r="K66" s="17"/>
     </row>
-    <row r="67" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="67" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="5">
         <v>46364.689583333333</v>
       </c>
@@ -3304,7 +3303,7 @@
       <c r="J67" s="17"/>
       <c r="K67" s="17"/>
     </row>
-    <row r="68" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="68" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -3335,7 +3334,7 @@
       <c r="J68" s="17"/>
       <c r="K68" s="17"/>
     </row>
-    <row r="69" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="69" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="5">
         <v>46251.688726851855</v>
       </c>
@@ -3366,7 +3365,7 @@
       <c r="J69" s="17"/>
       <c r="K69" s="17"/>
     </row>
-    <row r="70" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="70" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -3397,7 +3396,7 @@
       <c r="J70" s="17"/>
       <c r="K70" s="17"/>
     </row>
-    <row r="71" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="71" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -3428,7 +3427,7 @@
       <c r="J71" s="17"/>
       <c r="K71" s="17"/>
     </row>
-    <row r="72" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="72" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="5">
         <v>46251.688715277778</v>
       </c>
@@ -3461,7 +3460,7 @@
       </c>
       <c r="K72" s="17"/>
     </row>
-    <row r="73" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="73" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -3494,7 +3493,7 @@
       </c>
       <c r="K73" s="17"/>
     </row>
-    <row r="74" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="74" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -3527,7 +3526,7 @@
       </c>
       <c r="K74" s="17"/>
     </row>
-    <row r="75" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="75" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -3560,7 +3559,7 @@
       </c>
       <c r="K75" s="17"/>
     </row>
-    <row r="76" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="76" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="5">
         <v>46251.63554398148</v>
       </c>
@@ -3591,7 +3590,7 @@
       <c r="J76" s="17"/>
       <c r="K76" s="17"/>
     </row>
-    <row r="77" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="77" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="10" t="s">
         <v>85</v>
       </c>
@@ -3622,7 +3621,7 @@
       <c r="J77" s="17"/>
       <c r="K77" s="17"/>
     </row>
-    <row r="78" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="78" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="5">
         <v>46248.768750000003</v>
       </c>
@@ -3655,7 +3654,7 @@
       </c>
       <c r="K78" s="17"/>
     </row>
-    <row r="79" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="79" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="5">
         <v>46251.688715277778</v>
       </c>
@@ -3688,7 +3687,7 @@
       </c>
       <c r="K79" s="17"/>
     </row>
-    <row r="80" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="80" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="5">
         <v>46364.689583333333</v>
       </c>
@@ -3721,7 +3720,7 @@
       </c>
       <c r="K80" s="17"/>
     </row>
-    <row r="81" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="81" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="5">
         <v>46251.63554398148</v>
       </c>
@@ -3752,7 +3751,7 @@
       <c r="J81" s="17"/>
       <c r="K81" s="17"/>
     </row>
-    <row r="82" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="82" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -3783,7 +3782,7 @@
       <c r="J82" s="17"/>
       <c r="K82" s="17"/>
     </row>
-    <row r="83" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="83" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="5">
         <v>46251.688645833332</v>
       </c>
@@ -3814,7 +3813,7 @@
       <c r="J83" s="17"/>
       <c r="K83" s="17"/>
     </row>
-    <row r="84" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="84" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="5">
         <v>46251.635509259257</v>
       </c>
@@ -3845,7 +3844,7 @@
       <c r="J84" s="17"/>
       <c r="K84" s="17"/>
     </row>
-    <row r="85" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="85" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="5">
         <v>46248.768750000003</v>
       </c>
@@ -3876,7 +3875,7 @@
       <c r="J85" s="17"/>
       <c r="K85" s="17"/>
     </row>
-    <row r="86" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="86" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -3907,7 +3906,7 @@
       <c r="J86" s="17"/>
       <c r="K86" s="17"/>
     </row>
-    <row r="87" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="87" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -3938,7 +3937,7 @@
       <c r="J87" s="17"/>
       <c r="K87" s="17"/>
     </row>
-    <row r="88" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="88" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="5">
         <v>46251.688657407409</v>
       </c>
@@ -3971,7 +3970,7 @@
       </c>
       <c r="K88" s="17"/>
     </row>
-    <row r="89" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="89" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="5">
         <v>46245.635416666664</v>
       </c>
@@ -4002,7 +4001,7 @@
       <c r="J89" s="17"/>
       <c r="K89" s="17"/>
     </row>
-    <row r="90" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="90" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="7">
         <v>46248.768750000003</v>
       </c>
@@ -4035,7 +4034,7 @@
       </c>
       <c r="K90" s="17"/>
     </row>
-    <row r="91" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="91" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -4068,7 +4067,7 @@
       </c>
       <c r="K91" s="17"/>
     </row>
-    <row r="92" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="92" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="5">
         <v>46251.63554398148</v>
       </c>
@@ -4099,7 +4098,7 @@
       <c r="J92" s="17"/>
       <c r="K92" s="17"/>
     </row>
-    <row r="93" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="93" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -4132,7 +4131,7 @@
       </c>
       <c r="K93" s="17"/>
     </row>
-    <row r="94" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="94" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="5">
         <v>46251.635555555556</v>
       </c>
@@ -4163,7 +4162,7 @@
       <c r="J94" s="17"/>
       <c r="K94" s="17"/>
     </row>
-    <row r="95" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="95" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="5">
         <v>46251.635555555556</v>
       </c>
@@ -4196,7 +4195,7 @@
       </c>
       <c r="K95" s="17"/>
     </row>
-    <row r="96" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="96" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="5">
         <v>46251.688657407409</v>
       </c>
@@ -4227,7 +4226,7 @@
       <c r="J96" s="17"/>
       <c r="K96" s="17"/>
     </row>
-    <row r="97" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="97" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="5">
         <v>46251.688703703701</v>
       </c>
@@ -4260,7 +4259,7 @@
       </c>
       <c r="K97" s="17"/>
     </row>
-    <row r="98" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="98" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -4291,7 +4290,7 @@
       <c r="J98" s="17"/>
       <c r="K98" s="17"/>
     </row>
-    <row r="99" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="99" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="5">
         <v>46251.635509259257</v>
       </c>
@@ -4322,7 +4321,7 @@
       <c r="J99" s="17"/>
       <c r="K99" s="17"/>
     </row>
-    <row r="100" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="100" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="5">
         <v>46251.688692129632</v>
       </c>
@@ -4353,7 +4352,7 @@
       <c r="J100" s="17"/>
       <c r="K100" s="17"/>
     </row>
-    <row r="101" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="101" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="5">
         <v>46364.635416666664</v>
       </c>
@@ -4384,7 +4383,7 @@
       <c r="J101" s="17"/>
       <c r="K101" s="17"/>
     </row>
-    <row r="102" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="102" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="5">
         <v>46251.63554398148</v>
       </c>
@@ -4415,7 +4414,7 @@
       <c r="J102" s="17"/>
       <c r="K102" s="17"/>
     </row>
-    <row r="103" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="103" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -4446,7 +4445,7 @@
       <c r="J103" s="17"/>
       <c r="K103" s="17"/>
     </row>
-    <row r="104" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="104" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A104" s="5">
         <v>46251.688657407409</v>
       </c>
@@ -4477,7 +4476,7 @@
       <c r="J104" s="17"/>
       <c r="K104" s="17"/>
     </row>
-    <row r="105" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="105" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A105" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -4510,7 +4509,7 @@
       </c>
       <c r="K105" s="17"/>
     </row>
-    <row r="106" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="106" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A106" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -4543,7 +4542,7 @@
       </c>
       <c r="K106" s="17"/>
     </row>
-    <row r="107" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="107" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A107" s="5">
         <v>46247.645138888889</v>
       </c>
@@ -4574,7 +4573,7 @@
       <c r="J107" s="17"/>
       <c r="K107" s="17"/>
     </row>
-    <row r="108" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="108" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A108" s="7">
         <v>46248.768750000003</v>
       </c>
@@ -4605,7 +4604,7 @@
       <c r="J108" s="17"/>
       <c r="K108" s="17"/>
     </row>
-    <row r="109" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="109" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A109" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -4636,7 +4635,7 @@
       <c r="J109" s="17"/>
       <c r="K109" s="17"/>
     </row>
-    <row r="110" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="110" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A110" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -4667,7 +4666,7 @@
       <c r="J110" s="17"/>
       <c r="K110" s="17"/>
     </row>
-    <row r="111" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="111" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A111" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -4698,7 +4697,7 @@
       <c r="J111" s="17"/>
       <c r="K111" s="17"/>
     </row>
-    <row r="112" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="112" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A112" s="5">
         <v>46251.688703703701</v>
       </c>
@@ -4731,7 +4730,7 @@
       </c>
       <c r="K112" s="17"/>
     </row>
-    <row r="113" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="113" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A113" s="5">
         <v>46251.688715277778</v>
       </c>
@@ -4762,7 +4761,7 @@
       <c r="J113" s="17"/>
       <c r="K113" s="17"/>
     </row>
-    <row r="114" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="114" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A114" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -4793,7 +4792,7 @@
       <c r="J114" s="17"/>
       <c r="K114" s="17"/>
     </row>
-    <row r="115" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="115" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A115" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -4826,7 +4825,7 @@
       </c>
       <c r="K115" s="17"/>
     </row>
-    <row r="116" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="116" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A116" s="5">
         <v>46251.644641203704</v>
       </c>
@@ -4857,7 +4856,7 @@
       <c r="J116" s="17"/>
       <c r="K116" s="17"/>
     </row>
-    <row r="117" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="117" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A117" s="5">
         <v>46251.644652777781</v>
       </c>
@@ -4890,7 +4889,7 @@
       </c>
       <c r="K117" s="17"/>
     </row>
-    <row r="118" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="118" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A118" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -4923,7 +4922,7 @@
       </c>
       <c r="K118" s="17"/>
     </row>
-    <row r="119" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="119" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A119" s="5">
         <v>46251.644699074073</v>
       </c>
@@ -4954,7 +4953,7 @@
       <c r="J119" s="17"/>
       <c r="K119" s="17"/>
     </row>
-    <row r="120" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="120" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A120" s="5">
         <v>46251.644652777781</v>
       </c>
@@ -4985,7 +4984,7 @@
       <c r="J120" s="17"/>
       <c r="K120" s="17"/>
     </row>
-    <row r="121" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="121" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A121" s="5">
         <v>46247.645138888889</v>
       </c>
@@ -5016,7 +5015,7 @@
       <c r="J121" s="17"/>
       <c r="K121" s="17"/>
     </row>
-    <row r="122" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="122" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A122" s="5">
         <v>46251.644675925927</v>
       </c>
@@ -5047,7 +5046,7 @@
       <c r="J122" s="17"/>
       <c r="K122" s="17"/>
     </row>
-    <row r="123" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="123" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A123" s="5">
         <v>46251.644675925927</v>
       </c>
@@ -5078,7 +5077,7 @@
       <c r="J123" s="17"/>
       <c r="K123" s="17"/>
     </row>
-    <row r="124" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="124" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A124" s="5">
         <v>46251.644675925927</v>
       </c>
@@ -5109,7 +5108,7 @@
       <c r="J124" s="17"/>
       <c r="K124" s="17"/>
     </row>
-    <row r="125" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="125" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A125" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -5142,7 +5141,7 @@
       </c>
       <c r="K125" s="17"/>
     </row>
-    <row r="126" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="126" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A126" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -5173,7 +5172,7 @@
       <c r="J126" s="17"/>
       <c r="K126" s="17"/>
     </row>
-    <row r="127" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="127" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A127" s="5">
         <v>46251.644652777781</v>
       </c>
@@ -5204,7 +5203,7 @@
       <c r="J127" s="17"/>
       <c r="K127" s="17"/>
     </row>
-    <row r="128" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="128" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A128" s="5">
         <v>46246.689583333333</v>
       </c>
@@ -5237,7 +5236,7 @@
       </c>
       <c r="K128" s="17"/>
     </row>
-    <row r="129" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="129" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A129" s="5">
         <v>46251.688703703701</v>
       </c>
@@ -5270,7 +5269,7 @@
       </c>
       <c r="K129" s="17"/>
     </row>
-    <row r="130" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="130" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A130" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -5303,7 +5302,7 @@
       </c>
       <c r="K130" s="17"/>
     </row>
-    <row r="131" spans="1:11" ht="15" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="131" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A131" s="5">
         <v>46251.644675925927</v>
       </c>
@@ -5334,7 +5333,7 @@
       <c r="J131" s="17"/>
       <c r="K131" s="17"/>
     </row>
-    <row r="132" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="132" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A132" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -5367,7 +5366,7 @@
       </c>
       <c r="K132" s="17"/>
     </row>
-    <row r="133" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="133" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A133" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -5398,7 +5397,7 @@
       <c r="J133" s="17"/>
       <c r="K133" s="17"/>
     </row>
-    <row r="134" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="134" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A134" s="5">
         <v>46251.64466435185</v>
       </c>
@@ -5429,7 +5428,7 @@
       <c r="J134" s="17"/>
       <c r="K134" s="17"/>
     </row>
-    <row r="135" spans="1:11" ht="39" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="135" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A135" s="5">
         <v>46251.64466435185</v>
       </c>
@@ -5460,7 +5459,7 @@
       <c r="J135" s="17"/>
       <c r="K135" s="17"/>
     </row>
-    <row r="136" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="136" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A136" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -5493,7 +5492,7 @@
       </c>
       <c r="K136" s="17"/>
     </row>
-    <row r="137" spans="1:11" ht="26.5" hidden="1" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="137" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A137" s="5">
         <v>46251.644629629627</v>
       </c>
@@ -5524,7 +5523,7 @@
       <c r="J137" s="17"/>
       <c r="K137" s="17"/>
     </row>
-    <row r="138" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="138" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A138" s="5">
         <v>46251.644641203704</v>
       </c>
@@ -5555,7 +5554,7 @@
       <c r="J138" s="17"/>
       <c r="K138" s="17"/>
     </row>
-    <row r="139" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="139" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A139" s="5">
         <v>46251.64466435185</v>
       </c>
@@ -5586,7 +5585,7 @@
       <c r="J139" s="17"/>
       <c r="K139" s="17"/>
     </row>
-    <row r="140" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="140" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A140" s="5">
         <v>46251.688692129632</v>
       </c>
@@ -5648,7 +5647,7 @@
       <c r="J141" s="17"/>
       <c r="K141" s="17"/>
     </row>
-    <row r="142" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="142" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A142" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -5681,7 +5680,7 @@
       </c>
       <c r="K142" s="17"/>
     </row>
-    <row r="143" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="143" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A143" s="5">
         <v>46251.644641203704</v>
       </c>
@@ -5712,7 +5711,7 @@
       <c r="J143" s="17"/>
       <c r="K143" s="17"/>
     </row>
-    <row r="144" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="144" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A144" s="5">
         <v>46251.644675925927</v>
       </c>
@@ -5743,7 +5742,7 @@
       <c r="J144" s="17"/>
       <c r="K144" s="17"/>
     </row>
-    <row r="145" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="145" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A145" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -5809,7 +5808,7 @@
       </c>
       <c r="K146" s="17"/>
     </row>
-    <row r="147" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="147" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A147" s="5">
         <v>46251.688668981478</v>
       </c>
@@ -5842,7 +5841,7 @@
       </c>
       <c r="K147" s="17"/>
     </row>
-    <row r="148" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="148" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A148" s="5">
         <v>46251.688622685186</v>
       </c>
@@ -5875,7 +5874,7 @@
       </c>
       <c r="K148" s="17"/>
     </row>
-    <row r="149" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="149" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A149" s="5">
         <v>46251.688622685186</v>
       </c>
@@ -5908,7 +5907,7 @@
       </c>
       <c r="K149" s="17"/>
     </row>
-    <row r="150" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="150" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A150" s="5">
         <v>46251.644652777781</v>
       </c>
@@ -5941,7 +5940,7 @@
       </c>
       <c r="K150" s="17"/>
     </row>
-    <row r="151" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="151" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A151" s="5">
         <v>46251.64466435185</v>
       </c>
@@ -6003,7 +6002,7 @@
       <c r="J152" s="17"/>
       <c r="K152" s="17"/>
     </row>
-    <row r="153" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="153" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A153" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -6034,7 +6033,7 @@
       <c r="J153" s="17"/>
       <c r="K153" s="17"/>
     </row>
-    <row r="154" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="154" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A154" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -6131,7 +6130,7 @@
       <c r="J156" s="17"/>
       <c r="K156" s="17"/>
     </row>
-    <row r="157" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="157" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A157" s="5">
         <v>46251.644687499997</v>
       </c>
@@ -6162,7 +6161,7 @@
       <c r="J157" s="17"/>
       <c r="K157" s="17"/>
     </row>
-    <row r="158" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="158" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A158" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -6193,7 +6192,7 @@
       <c r="J158" s="17"/>
       <c r="K158" s="17"/>
     </row>
-    <row r="159" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="159" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A159" s="5">
         <v>46251.688715277778</v>
       </c>
@@ -6224,7 +6223,7 @@
       <c r="J159" s="17"/>
       <c r="K159" s="17"/>
     </row>
-    <row r="160" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="160" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A160" s="5">
         <v>46251.688622685186</v>
       </c>
@@ -6257,7 +6256,7 @@
       </c>
       <c r="K160" s="17"/>
     </row>
-    <row r="161" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="161" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A161" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -6288,7 +6287,7 @@
       <c r="J161" s="17"/>
       <c r="K161" s="17"/>
     </row>
-    <row r="162" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="162" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A162" s="5">
         <v>46251.688692129632</v>
       </c>
@@ -6319,7 +6318,7 @@
       <c r="J162" s="17"/>
       <c r="K162" s="17"/>
     </row>
-    <row r="163" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="163" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A163" s="5">
         <v>46251.635578703703</v>
       </c>
@@ -6385,7 +6384,7 @@
       </c>
       <c r="K164" s="17"/>
     </row>
-    <row r="165" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="165" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A165" s="5">
         <v>46251.688611111109</v>
       </c>
@@ -6416,7 +6415,7 @@
       <c r="J165" s="17"/>
       <c r="K165" s="17"/>
     </row>
-    <row r="166" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="166" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A166" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -6447,7 +6446,7 @@
       <c r="J166" s="17"/>
       <c r="K166" s="17"/>
     </row>
-    <row r="167" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="167" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A167" s="5">
         <v>46251.635520833333</v>
       </c>
@@ -6478,7 +6477,7 @@
       <c r="J167" s="17"/>
       <c r="K167" s="17"/>
     </row>
-    <row r="168" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="168" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A168" s="5">
         <v>46251.635555555556</v>
       </c>
@@ -6509,7 +6508,7 @@
       <c r="J168" s="17"/>
       <c r="K168" s="17"/>
     </row>
-    <row r="169" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="169" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A169" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -6540,7 +6539,7 @@
       <c r="J169" s="17"/>
       <c r="K169" s="17"/>
     </row>
-    <row r="170" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="170" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A170" s="5">
         <v>46251.63553240741</v>
       </c>
@@ -6571,7 +6570,7 @@
       <c r="J170" s="17"/>
       <c r="K170" s="17"/>
     </row>
-    <row r="171" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="171" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A171" s="5">
         <v>46248.770833333336</v>
       </c>
@@ -6604,7 +6603,7 @@
       </c>
       <c r="K171" s="17"/>
     </row>
-    <row r="172" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="172" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A172" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -6635,7 +6634,7 @@
       <c r="J172" s="17"/>
       <c r="K172" s="17"/>
     </row>
-    <row r="173" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="173" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A173" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -6666,7 +6665,7 @@
       <c r="J173" s="17"/>
       <c r="K173" s="17"/>
     </row>
-    <row r="174" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="174" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A174" s="5">
         <v>46364.635416666664</v>
       </c>
@@ -6697,7 +6696,7 @@
       <c r="J174" s="17"/>
       <c r="K174" s="17"/>
     </row>
-    <row r="175" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="175" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A175" s="5">
         <v>46248.635416666664</v>
       </c>
@@ -6730,7 +6729,7 @@
       </c>
       <c r="K175" s="17"/>
     </row>
-    <row r="176" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="176" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A176" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -6761,7 +6760,7 @@
       <c r="J176" s="17"/>
       <c r="K176" s="17"/>
     </row>
-    <row r="177" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="177" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A177" s="10" t="s">
         <v>85</v>
       </c>
@@ -6858,7 +6857,7 @@
       </c>
       <c r="K179" s="17"/>
     </row>
-    <row r="180" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="180" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A180" s="5">
         <v>46251.688668981478</v>
       </c>
@@ -6922,7 +6921,7 @@
       <c r="J181" s="17"/>
       <c r="K181" s="17"/>
     </row>
-    <row r="182" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="182" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A182" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -6984,7 +6983,7 @@
       <c r="J183" s="17"/>
       <c r="K183" s="17"/>
     </row>
-    <row r="184" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="184" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A184" s="5">
         <v>46251.635555555556</v>
       </c>
@@ -7015,7 +7014,7 @@
       <c r="J184" s="17"/>
       <c r="K184" s="17"/>
     </row>
-    <row r="185" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="185" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A185" s="26">
         <v>46251.688634259262</v>
       </c>
@@ -7048,7 +7047,7 @@
       </c>
       <c r="K185" s="17"/>
     </row>
-    <row r="186" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="186" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A186" s="5">
         <v>46364.635416666664</v>
       </c>
@@ -7079,7 +7078,7 @@
       <c r="J186" s="17"/>
       <c r="K186" s="17"/>
     </row>
-    <row r="187" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="187" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A187" s="5">
         <v>46251.635567129626</v>
       </c>
@@ -7143,7 +7142,7 @@
       </c>
       <c r="K188" s="17"/>
     </row>
-    <row r="189" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="189" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A189" s="5">
         <v>46251.688692129632</v>
       </c>
@@ -7174,7 +7173,7 @@
       <c r="J189" s="17"/>
       <c r="K189" s="17"/>
     </row>
-    <row r="190" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="190" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A190" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -7207,7 +7206,7 @@
       </c>
       <c r="K190" s="17"/>
     </row>
-    <row r="191" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="191" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A191" s="5">
         <v>46246.635416666664</v>
       </c>
@@ -7238,7 +7237,7 @@
       <c r="J191" s="17"/>
       <c r="K191" s="17"/>
     </row>
-    <row r="192" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="192" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A192" s="5">
         <v>46239.635416666664</v>
       </c>
@@ -7269,7 +7268,7 @@
       <c r="J192" s="17"/>
       <c r="K192" s="17"/>
     </row>
-    <row r="193" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="193" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A193" s="31">
         <v>46251.688634259262</v>
       </c>
@@ -7302,7 +7301,7 @@
       </c>
       <c r="K193" s="17"/>
     </row>
-    <row r="194" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="194" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A194" s="5">
         <v>46211.635416666664</v>
       </c>
@@ -7366,7 +7365,7 @@
       </c>
       <c r="K195" s="17"/>
     </row>
-    <row r="196" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="196" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A196" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -7397,7 +7396,7 @@
       <c r="J196" s="17"/>
       <c r="K196" s="17"/>
     </row>
-    <row r="197" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="197" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A197" s="5">
         <v>46303.635416666664</v>
       </c>
@@ -7428,7 +7427,7 @@
       <c r="J197" s="17"/>
       <c r="K197" s="17"/>
     </row>
-    <row r="198" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="198" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A198" s="5">
         <v>46251.688576388886</v>
       </c>
@@ -7459,7 +7458,7 @@
       <c r="J198" s="17"/>
       <c r="K198" s="17"/>
     </row>
-    <row r="199" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="199" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A199" s="5">
         <v>46211.635416666664</v>
       </c>
@@ -7523,7 +7522,7 @@
       </c>
       <c r="K200" s="17"/>
     </row>
-    <row r="201" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="201" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A201" s="10" t="s">
         <v>85</v>
       </c>
@@ -7554,7 +7553,7 @@
       <c r="J201" s="17"/>
       <c r="K201" s="17"/>
     </row>
-    <row r="202" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="202" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A202" s="5">
         <v>46245.693055555559</v>
       </c>
@@ -7618,7 +7617,7 @@
       </c>
       <c r="K203" s="17"/>
     </row>
-    <row r="204" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="204" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A204" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -7649,7 +7648,7 @@
       <c r="J204" s="17"/>
       <c r="K204" s="17"/>
     </row>
-    <row r="205" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="205" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A205" s="5">
         <v>46241.635416666664</v>
       </c>
@@ -7680,7 +7679,7 @@
       <c r="J205" s="17"/>
       <c r="K205" s="17"/>
     </row>
-    <row r="206" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="206" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A206" s="5">
         <v>46246.689583333333</v>
       </c>
@@ -7711,7 +7710,7 @@
       <c r="J206" s="17"/>
       <c r="K206" s="17"/>
     </row>
-    <row r="207" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="207" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A207" s="5">
         <v>46247.635416666664</v>
       </c>
@@ -7742,7 +7741,7 @@
       <c r="J207" s="17"/>
       <c r="K207" s="17"/>
     </row>
-    <row r="208" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="208" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A208" s="10" t="s">
         <v>85</v>
       </c>
@@ -7773,7 +7772,7 @@
       <c r="J208" s="17"/>
       <c r="K208" s="17"/>
     </row>
-    <row r="209" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="209" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A209" s="5">
         <v>46211.635416666664</v>
       </c>
@@ -7835,7 +7834,7 @@
       <c r="J210" s="17"/>
       <c r="K210" s="17"/>
     </row>
-    <row r="211" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="211" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A211" s="5">
         <v>46244.635416666664</v>
       </c>
@@ -7866,7 +7865,7 @@
       <c r="J211" s="17"/>
       <c r="K211" s="17"/>
     </row>
-    <row r="212" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="212" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A212" s="5">
         <v>46364.689583333333</v>
       </c>
@@ -7930,7 +7929,7 @@
       </c>
       <c r="K213" s="17"/>
     </row>
-    <row r="214" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="214" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A214" s="10" t="s">
         <v>85</v>
       </c>
@@ -7994,7 +7993,7 @@
       </c>
       <c r="K215" s="17"/>
     </row>
-    <row r="216" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="216" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A216" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -8025,7 +8024,7 @@
       <c r="J216" s="17"/>
       <c r="K216" s="17"/>
     </row>
-    <row r="217" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="217" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A217" s="10" t="s">
         <v>85</v>
       </c>
@@ -8089,7 +8088,7 @@
       </c>
       <c r="K218" s="17"/>
     </row>
-    <row r="219" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="219" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A219" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -8120,7 +8119,7 @@
       <c r="J219" s="17"/>
       <c r="K219" s="17"/>
     </row>
-    <row r="220" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="220" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A220" s="10" t="s">
         <v>85</v>
       </c>
@@ -8151,7 +8150,7 @@
       <c r="J220" s="17"/>
       <c r="K220" s="17"/>
     </row>
-    <row r="221" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="221" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A221" s="2">
         <v>46251.688634259262</v>
       </c>
@@ -8215,7 +8214,7 @@
       <c r="J222" s="17"/>
       <c r="K222" s="17"/>
     </row>
-    <row r="223" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="223" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A223" s="5">
         <v>46211.635416666664</v>
       </c>
@@ -8246,7 +8245,7 @@
       <c r="J223" s="17"/>
       <c r="K223" s="17"/>
     </row>
-    <row r="224" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="224" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A224" s="5">
         <v>46239.788888888892</v>
       </c>
@@ -8277,7 +8276,7 @@
       <c r="J224" s="17"/>
       <c r="K224" s="17"/>
     </row>
-    <row r="225" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="225" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A225" s="5">
         <v>46247.645138888889</v>
       </c>
@@ -8341,7 +8340,7 @@
       </c>
       <c r="K226" s="17"/>
     </row>
-    <row r="227" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="227" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A227" s="10" t="s">
         <v>85</v>
       </c>
@@ -8372,7 +8371,7 @@
       <c r="J227" s="17"/>
       <c r="K227" s="17"/>
     </row>
-    <row r="228" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="228" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A228" s="5">
         <v>46150.788888888892</v>
       </c>
@@ -8403,7 +8402,7 @@
       <c r="J228" s="17"/>
       <c r="K228" s="17"/>
     </row>
-    <row r="229" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="229" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A229" s="34">
         <v>46251.688634259262</v>
       </c>
@@ -8436,7 +8435,7 @@
       </c>
       <c r="K229" s="17"/>
     </row>
-    <row r="230" spans="1:11" ht="39" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="230" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A230" s="14">
         <v>46334.645833333336</v>
       </c>
@@ -8467,7 +8466,7 @@
       <c r="J230" s="17"/>
       <c r="K230" s="17"/>
     </row>
-    <row r="231" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="231" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A231" s="5">
         <v>46251.688634259262</v>
       </c>
@@ -8500,7 +8499,7 @@
       </c>
       <c r="K231" s="17"/>
     </row>
-    <row r="232" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="232" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A232" s="5">
         <v>46364.689583333333</v>
       </c>
@@ -8533,7 +8532,7 @@
       </c>
       <c r="K232" s="17"/>
     </row>
-    <row r="233" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="233" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A233" s="5">
         <v>46251.688634259262</v>
       </c>
@@ -8566,7 +8565,7 @@
       </c>
       <c r="K233" s="17"/>
     </row>
-    <row r="234" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="234" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A234" s="5">
         <v>46246.689583333333</v>
       </c>
@@ -8599,7 +8598,7 @@
       </c>
       <c r="K234" s="17"/>
     </row>
-    <row r="235" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="235" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A235" s="5">
         <v>46251.688634259262</v>
       </c>
@@ -8632,7 +8631,7 @@
       </c>
       <c r="K235" s="17"/>
     </row>
-    <row r="236" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="236" spans="1:11" ht="16" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A236" s="5">
         <v>46247.689583333333</v>
       </c>
@@ -8665,7 +8664,7 @@
       </c>
       <c r="K236" s="17"/>
     </row>
-    <row r="237" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="237" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A237" s="6" t="s">
         <v>190</v>
       </c>
@@ -8698,7 +8697,7 @@
       </c>
       <c r="K237" s="17"/>
     </row>
-    <row r="238" spans="1:11" ht="26.5" thickBot="1" x14ac:dyDescent="0.4">
+    <row r="238" spans="1:11" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A238" s="5">
         <v>46239.793055555558</v>
       </c>
@@ -8730,16 +8729,6 @@
       <c r="K238" s="17"/>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K238" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="2">
-      <filters>
-        <filter val="S"/>
-      </filters>
-    </filterColumn>
-    <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A2:K238">
-      <sortCondition ref="F1"/>
-    </sortState>
-  </autoFilter>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
@@ -15971,7 +15960,7 @@
         <v>120</v>
       </c>
       <c r="P2" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B2, $C$2:$C$970, C2, $D$2:$D$970, D2, $E$2:$E$970, E2) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="P2:P65" si="0">IF(COUNTIFS( $B$2:$B$970, B2, $C$2:$C$970, C2, $D$2:$D$970, D2, $E$2:$E$970, E2) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -15996,7 +15985,7 @@
       </c>
       <c r="N3"/>
       <c r="P3" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B3, $C$2:$C$970, C3, $D$2:$D$970, D3, $E$2:$E$970, E3) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16021,7 +16010,7 @@
       </c>
       <c r="N4"/>
       <c r="P4" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B4, $C$2:$C$970, C4, $D$2:$D$970, D4, $E$2:$E$970, E4) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16048,7 +16037,7 @@
         <v>125</v>
       </c>
       <c r="P5" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B5, $C$2:$C$970, C5, $D$2:$D$970, D5, $E$2:$E$970, E5) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16075,7 +16064,7 @@
         <v>117</v>
       </c>
       <c r="P6" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B6, $C$2:$C$970, C6, $D$2:$D$970, D6, $E$2:$E$970, E6) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16102,7 +16091,7 @@
         <v>119</v>
       </c>
       <c r="P7" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B7, $C$2:$C$970, C7, $D$2:$D$970, D7, $E$2:$E$970, E7) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16129,7 +16118,7 @@
         <v>120</v>
       </c>
       <c r="P8" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B8, $C$2:$C$970, C8, $D$2:$D$970, D8, $E$2:$E$970, E8) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16156,7 +16145,7 @@
         <v>117</v>
       </c>
       <c r="P9" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B9, $C$2:$C$970, C9, $D$2:$D$970, D9, $E$2:$E$970, E9) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16183,7 +16172,7 @@
         <v>119</v>
       </c>
       <c r="P10" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B10, $C$2:$C$970, C10, $D$2:$D$970, D10, $E$2:$E$970, E10) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16210,7 +16199,7 @@
         <v>119</v>
       </c>
       <c r="P11" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B11, $C$2:$C$970, C11, $D$2:$D$970, D11, $E$2:$E$970, E11) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16237,7 +16226,7 @@
         <v>117</v>
       </c>
       <c r="P12" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B12, $C$2:$C$970, C12, $D$2:$D$970, D12, $E$2:$E$970, E12) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16264,7 +16253,7 @@
         <v>117</v>
       </c>
       <c r="P13" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B13, $C$2:$C$970, C13, $D$2:$D$970, D13, $E$2:$E$970, E13) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16291,7 +16280,7 @@
         <v>120</v>
       </c>
       <c r="P14" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B14, $C$2:$C$970, C14, $D$2:$D$970, D14, $E$2:$E$970, E14) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16318,7 +16307,7 @@
         <v>123</v>
       </c>
       <c r="P15" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B15, $C$2:$C$970, C15, $D$2:$D$970, D15, $E$2:$E$970, E15) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16343,7 +16332,7 @@
       </c>
       <c r="N16"/>
       <c r="P16" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B16, $C$2:$C$970, C16, $D$2:$D$970, D16, $E$2:$E$970, E16) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16370,7 +16359,7 @@
         <v>123</v>
       </c>
       <c r="P17" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B17, $C$2:$C$970, C17, $D$2:$D$970, D17, $E$2:$E$970, E17) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16397,7 +16386,7 @@
         <v>123</v>
       </c>
       <c r="P18" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B18, $C$2:$C$970, C18, $D$2:$D$970, D18, $E$2:$E$970, E18) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16424,7 +16413,7 @@
         <v>120</v>
       </c>
       <c r="P19" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B19, $C$2:$C$970, C19, $D$2:$D$970, D19, $E$2:$E$970, E19) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16451,7 +16440,7 @@
         <v>122</v>
       </c>
       <c r="P20" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B20, $C$2:$C$970, C20, $D$2:$D$970, D20, $E$2:$E$970, E20) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16478,7 +16467,7 @@
         <v>120</v>
       </c>
       <c r="P21" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B21, $C$2:$C$970, C21, $D$2:$D$970, D21, $E$2:$E$970, E21) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16505,7 +16494,7 @@
         <v>120</v>
       </c>
       <c r="P22" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B22, $C$2:$C$970, C22, $D$2:$D$970, D22, $E$2:$E$970, E22) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16532,7 +16521,7 @@
         <v>121</v>
       </c>
       <c r="P23" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B23, $C$2:$C$970, C23, $D$2:$D$970, D23, $E$2:$E$970, E23) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16557,7 +16546,7 @@
       </c>
       <c r="N24"/>
       <c r="P24" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B24, $C$2:$C$970, C24, $D$2:$D$970, D24, $E$2:$E$970, E24) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16584,7 +16573,7 @@
         <v>121</v>
       </c>
       <c r="P25" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B25, $C$2:$C$970, C25, $D$2:$D$970, D25, $E$2:$E$970, E25) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16609,7 +16598,7 @@
       </c>
       <c r="N26"/>
       <c r="P26" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B26, $C$2:$C$970, C26, $D$2:$D$970, D26, $E$2:$E$970, E26) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16634,7 +16623,7 @@
       </c>
       <c r="N27"/>
       <c r="P27" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B27, $C$2:$C$970, C27, $D$2:$D$970, D27, $E$2:$E$970, E27) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16661,7 +16650,7 @@
         <v>121</v>
       </c>
       <c r="P28" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B28, $C$2:$C$970, C28, $D$2:$D$970, D28, $E$2:$E$970, E28) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16688,7 +16677,7 @@
         <v>121</v>
       </c>
       <c r="P29" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B29, $C$2:$C$970, C29, $D$2:$D$970, D29, $E$2:$E$970, E29) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16715,7 +16704,7 @@
         <v>123</v>
       </c>
       <c r="P30" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B30, $C$2:$C$970, C30, $D$2:$D$970, D30, $E$2:$E$970, E30) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16742,7 +16731,7 @@
         <v>121</v>
       </c>
       <c r="P31" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B31, $C$2:$C$970, C31, $D$2:$D$970, D31, $E$2:$E$970, E31) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16767,7 +16756,7 @@
       </c>
       <c r="N32"/>
       <c r="P32" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B32, $C$2:$C$970, C32, $D$2:$D$970, D32, $E$2:$E$970, E32) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16792,7 +16781,7 @@
       </c>
       <c r="N33"/>
       <c r="P33" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B33, $C$2:$C$970, C33, $D$2:$D$970, D33, $E$2:$E$970, E33) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16817,7 +16806,7 @@
       </c>
       <c r="N34"/>
       <c r="P34" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B34, $C$2:$C$970, C34, $D$2:$D$970, D34, $E$2:$E$970, E34) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16844,7 +16833,7 @@
         <v>125</v>
       </c>
       <c r="P35" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B35, $C$2:$C$970, C35, $D$2:$D$970, D35, $E$2:$E$970, E35) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16869,7 +16858,7 @@
       </c>
       <c r="N36"/>
       <c r="P36" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B36, $C$2:$C$970, C36, $D$2:$D$970, D36, $E$2:$E$970, E36) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16894,7 +16883,7 @@
       </c>
       <c r="N37"/>
       <c r="P37" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B37, $C$2:$C$970, C37, $D$2:$D$970, D37, $E$2:$E$970, E37) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16921,7 +16910,7 @@
         <v>121</v>
       </c>
       <c r="P38" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B38, $C$2:$C$970, C38, $D$2:$D$970, D38, $E$2:$E$970, E38) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16948,7 +16937,7 @@
         <v>123</v>
       </c>
       <c r="P39" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B39, $C$2:$C$970, C39, $D$2:$D$970, D39, $E$2:$E$970, E39) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -16975,7 +16964,7 @@
         <v>120</v>
       </c>
       <c r="P40" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B40, $C$2:$C$970, C40, $D$2:$D$970, D40, $E$2:$E$970, E40) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17002,7 +16991,7 @@
         <v>120</v>
       </c>
       <c r="P41" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B41, $C$2:$C$970, C41, $D$2:$D$970, D41, $E$2:$E$970, E41) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17027,7 +17016,7 @@
       </c>
       <c r="N42"/>
       <c r="P42" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B42, $C$2:$C$970, C42, $D$2:$D$970, D42, $E$2:$E$970, E42) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17054,7 +17043,7 @@
         <v>124</v>
       </c>
       <c r="P43" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B43, $C$2:$C$970, C43, $D$2:$D$970, D43, $E$2:$E$970, E43) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17079,7 +17068,7 @@
       </c>
       <c r="N44"/>
       <c r="P44" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B44, $C$2:$C$970, C44, $D$2:$D$970, D44, $E$2:$E$970, E44) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17106,7 +17095,7 @@
         <v>122</v>
       </c>
       <c r="P45" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B45, $C$2:$C$970, C45, $D$2:$D$970, D45, $E$2:$E$970, E45) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17131,7 +17120,7 @@
       </c>
       <c r="N46"/>
       <c r="P46" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B46, $C$2:$C$970, C46, $D$2:$D$970, D46, $E$2:$E$970, E46) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17158,7 +17147,7 @@
         <v>124</v>
       </c>
       <c r="P47" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B47, $C$2:$C$970, C47, $D$2:$D$970, D47, $E$2:$E$970, E47) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17183,7 +17172,7 @@
       </c>
       <c r="N48"/>
       <c r="P48" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B48, $C$2:$C$970, C48, $D$2:$D$970, D48, $E$2:$E$970, E48) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17208,7 +17197,7 @@
       </c>
       <c r="N49"/>
       <c r="P49" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B49, $C$2:$C$970, C49, $D$2:$D$970, D49, $E$2:$E$970, E49) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17233,7 +17222,7 @@
       </c>
       <c r="N50"/>
       <c r="P50" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B50, $C$2:$C$970, C50, $D$2:$D$970, D50, $E$2:$E$970, E50) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17258,7 +17247,7 @@
       </c>
       <c r="N51"/>
       <c r="P51" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B51, $C$2:$C$970, C51, $D$2:$D$970, D51, $E$2:$E$970, E51) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17285,7 +17274,7 @@
         <v>120</v>
       </c>
       <c r="P52" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B52, $C$2:$C$970, C52, $D$2:$D$970, D52, $E$2:$E$970, E52) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17312,7 +17301,7 @@
         <v>122</v>
       </c>
       <c r="P53" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B53, $C$2:$C$970, C53, $D$2:$D$970, D53, $E$2:$E$970, E53) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17339,7 +17328,7 @@
         <v>124</v>
       </c>
       <c r="P54" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B54, $C$2:$C$970, C54, $D$2:$D$970, D54, $E$2:$E$970, E54) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17364,7 +17353,7 @@
       </c>
       <c r="N55"/>
       <c r="P55" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B55, $C$2:$C$970, C55, $D$2:$D$970, D55, $E$2:$E$970, E55) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17391,7 +17380,7 @@
         <v>122</v>
       </c>
       <c r="P56" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B56, $C$2:$C$970, C56, $D$2:$D$970, D56, $E$2:$E$970, E56) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17416,7 +17405,7 @@
       </c>
       <c r="N57"/>
       <c r="P57" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B57, $C$2:$C$970, C57, $D$2:$D$970, D57, $E$2:$E$970, E57) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17441,7 +17430,7 @@
       </c>
       <c r="N58"/>
       <c r="P58" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B58, $C$2:$C$970, C58, $D$2:$D$970, D58, $E$2:$E$970, E58) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17466,7 +17455,7 @@
       </c>
       <c r="N59"/>
       <c r="P59" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B59, $C$2:$C$970, C59, $D$2:$D$970, D59, $E$2:$E$970, E59) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17491,7 +17480,7 @@
       </c>
       <c r="N60"/>
       <c r="P60" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B60, $C$2:$C$970, C60, $D$2:$D$970, D60, $E$2:$E$970, E60) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17518,7 +17507,7 @@
         <v>123</v>
       </c>
       <c r="P61" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B61, $C$2:$C$970, C61, $D$2:$D$970, D61, $E$2:$E$970, E61) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17545,7 +17534,7 @@
         <v>120</v>
       </c>
       <c r="P62" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B62, $C$2:$C$970, C62, $D$2:$D$970, D62, $E$2:$E$970, E62) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17572,7 +17561,7 @@
         <v>120</v>
       </c>
       <c r="P63" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B63, $C$2:$C$970, C63, $D$2:$D$970, D63, $E$2:$E$970, E63) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17599,7 +17588,7 @@
         <v>120</v>
       </c>
       <c r="P64" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B64, $C$2:$C$970, C64, $D$2:$D$970, D64, $E$2:$E$970, E64) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17626,7 +17615,7 @@
         <v>125</v>
       </c>
       <c r="P65" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B65, $C$2:$C$970, C65, $D$2:$D$970, D65, $E$2:$E$970, E65) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="0"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17651,7 +17640,7 @@
       </c>
       <c r="N66"/>
       <c r="P66" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B66, $C$2:$C$970, C66, $D$2:$D$970, D66, $E$2:$E$970, E66) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="P66:P129" si="1">IF(COUNTIFS( $B$2:$B$970, B66, $C$2:$C$970, C66, $D$2:$D$970, D66, $E$2:$E$970, E66) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -17676,7 +17665,7 @@
       </c>
       <c r="N67"/>
       <c r="P67" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B67, $C$2:$C$970, C67, $D$2:$D$970, D67, $E$2:$E$970, E67) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17701,7 +17690,7 @@
       </c>
       <c r="N68"/>
       <c r="P68" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B68, $C$2:$C$970, C68, $D$2:$D$970, D68, $E$2:$E$970, E68) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17728,7 +17717,7 @@
         <v>125</v>
       </c>
       <c r="P69" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B69, $C$2:$C$970, C69, $D$2:$D$970, D69, $E$2:$E$970, E69) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17753,7 +17742,7 @@
       </c>
       <c r="N70"/>
       <c r="P70" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B70, $C$2:$C$970, C70, $D$2:$D$970, D70, $E$2:$E$970, E70) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17778,7 +17767,7 @@
       </c>
       <c r="N71"/>
       <c r="P71" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B71, $C$2:$C$970, C71, $D$2:$D$970, D71, $E$2:$E$970, E71) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17803,7 +17792,7 @@
       </c>
       <c r="N72"/>
       <c r="P72" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B72, $C$2:$C$970, C72, $D$2:$D$970, D72, $E$2:$E$970, E72) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17828,7 +17817,7 @@
       </c>
       <c r="N73"/>
       <c r="P73" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B73, $C$2:$C$970, C73, $D$2:$D$970, D73, $E$2:$E$970, E73) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17853,7 +17842,7 @@
       </c>
       <c r="N74"/>
       <c r="P74" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B74, $C$2:$C$970, C74, $D$2:$D$970, D74, $E$2:$E$970, E74) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17878,7 +17867,7 @@
       </c>
       <c r="N75"/>
       <c r="P75" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B75, $C$2:$C$970, C75, $D$2:$D$970, D75, $E$2:$E$970, E75) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17905,7 +17894,7 @@
         <v>125</v>
       </c>
       <c r="P76" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B76, $C$2:$C$970, C76, $D$2:$D$970, D76, $E$2:$E$970, E76) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17930,7 +17919,7 @@
       </c>
       <c r="N77"/>
       <c r="P77" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B77, $C$2:$C$970, C77, $D$2:$D$970, D77, $E$2:$E$970, E77) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17955,7 +17944,7 @@
       </c>
       <c r="N78"/>
       <c r="P78" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B78, $C$2:$C$970, C78, $D$2:$D$970, D78, $E$2:$E$970, E78) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -17982,7 +17971,7 @@
         <v>125</v>
       </c>
       <c r="P79" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B79, $C$2:$C$970, C79, $D$2:$D$970, D79, $E$2:$E$970, E79) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18007,7 +17996,7 @@
       </c>
       <c r="N80"/>
       <c r="P80" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B80, $C$2:$C$970, C80, $D$2:$D$970, D80, $E$2:$E$970, E80) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18032,7 +18021,7 @@
       </c>
       <c r="N81"/>
       <c r="P81" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B81, $C$2:$C$970, C81, $D$2:$D$970, D81, $E$2:$E$970, E81) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18057,7 +18046,7 @@
       </c>
       <c r="N82"/>
       <c r="P82" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B82, $C$2:$C$970, C82, $D$2:$D$970, D82, $E$2:$E$970, E82) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18082,7 +18071,7 @@
       </c>
       <c r="N83"/>
       <c r="P83" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B83, $C$2:$C$970, C83, $D$2:$D$970, D83, $E$2:$E$970, E83) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18107,7 +18096,7 @@
       </c>
       <c r="N84"/>
       <c r="P84" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B84, $C$2:$C$970, C84, $D$2:$D$970, D84, $E$2:$E$970, E84) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18132,7 +18121,7 @@
       </c>
       <c r="N85"/>
       <c r="P85" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B85, $C$2:$C$970, C85, $D$2:$D$970, D85, $E$2:$E$970, E85) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18157,7 +18146,7 @@
       </c>
       <c r="N86"/>
       <c r="P86" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B86, $C$2:$C$970, C86, $D$2:$D$970, D86, $E$2:$E$970, E86) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18182,7 +18171,7 @@
       </c>
       <c r="N87"/>
       <c r="P87" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B87, $C$2:$C$970, C87, $D$2:$D$970, D87, $E$2:$E$970, E87) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18207,7 +18196,7 @@
       </c>
       <c r="N88"/>
       <c r="P88" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B88, $C$2:$C$970, C88, $D$2:$D$970, D88, $E$2:$E$970, E88) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18232,7 +18221,7 @@
       </c>
       <c r="N89"/>
       <c r="P89" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B89, $C$2:$C$970, C89, $D$2:$D$970, D89, $E$2:$E$970, E89) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18257,7 +18246,7 @@
       </c>
       <c r="N90"/>
       <c r="P90" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B90, $C$2:$C$970, C90, $D$2:$D$970, D90, $E$2:$E$970, E90) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18282,7 +18271,7 @@
       </c>
       <c r="N91"/>
       <c r="P91" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B91, $C$2:$C$970, C91, $D$2:$D$970, D91, $E$2:$E$970, E91) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18307,7 +18296,7 @@
       </c>
       <c r="N92"/>
       <c r="P92" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B92, $C$2:$C$970, C92, $D$2:$D$970, D92, $E$2:$E$970, E92) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18332,7 +18321,7 @@
       </c>
       <c r="N93"/>
       <c r="P93" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B93, $C$2:$C$970, C93, $D$2:$D$970, D93, $E$2:$E$970, E93) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18357,7 +18346,7 @@
       </c>
       <c r="N94"/>
       <c r="P94" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B94, $C$2:$C$970, C94, $D$2:$D$970, D94, $E$2:$E$970, E94) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18382,7 +18371,7 @@
       </c>
       <c r="N95"/>
       <c r="P95" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B95, $C$2:$C$970, C95, $D$2:$D$970, D95, $E$2:$E$970, E95) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18407,7 +18396,7 @@
       </c>
       <c r="N96"/>
       <c r="P96" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B96, $C$2:$C$970, C96, $D$2:$D$970, D96, $E$2:$E$970, E96) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18432,7 +18421,7 @@
       </c>
       <c r="N97"/>
       <c r="P97" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B97, $C$2:$C$970, C97, $D$2:$D$970, D97, $E$2:$E$970, E97) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18457,7 +18446,7 @@
       </c>
       <c r="N98"/>
       <c r="P98" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B98, $C$2:$C$970, C98, $D$2:$D$970, D98, $E$2:$E$970, E98) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18482,7 +18471,7 @@
       </c>
       <c r="N99"/>
       <c r="P99" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B99, $C$2:$C$970, C99, $D$2:$D$970, D99, $E$2:$E$970, E99) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18507,7 +18496,7 @@
       </c>
       <c r="N100"/>
       <c r="P100" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B100, $C$2:$C$970, C100, $D$2:$D$970, D100, $E$2:$E$970, E100) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18534,7 +18523,7 @@
         <v>120</v>
       </c>
       <c r="P101" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B101, $C$2:$C$970, C101, $D$2:$D$970, D101, $E$2:$E$970, E101) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18559,7 +18548,7 @@
       </c>
       <c r="N102"/>
       <c r="P102" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B102, $C$2:$C$970, C102, $D$2:$D$970, D102, $E$2:$E$970, E102) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18584,7 +18573,7 @@
       </c>
       <c r="N103"/>
       <c r="P103" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B103, $C$2:$C$970, C103, $D$2:$D$970, D103, $E$2:$E$970, E103) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18609,7 +18598,7 @@
       </c>
       <c r="N104"/>
       <c r="P104" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B104, $C$2:$C$970, C104, $D$2:$D$970, D104, $E$2:$E$970, E104) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18634,7 +18623,7 @@
       </c>
       <c r="N105"/>
       <c r="P105" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B105, $C$2:$C$970, C105, $D$2:$D$970, D105, $E$2:$E$970, E105) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18659,7 +18648,7 @@
       </c>
       <c r="N106"/>
       <c r="P106" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B106, $C$2:$C$970, C106, $D$2:$D$970, D106, $E$2:$E$970, E106) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18684,7 +18673,7 @@
       </c>
       <c r="N107"/>
       <c r="P107" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B107, $C$2:$C$970, C107, $D$2:$D$970, D107, $E$2:$E$970, E107) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18709,7 +18698,7 @@
       </c>
       <c r="N108"/>
       <c r="P108" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B108, $C$2:$C$970, C108, $D$2:$D$970, D108, $E$2:$E$970, E108) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18736,7 +18725,7 @@
         <v>120</v>
       </c>
       <c r="P109" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B109, $C$2:$C$970, C109, $D$2:$D$970, D109, $E$2:$E$970, E109) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18761,7 +18750,7 @@
       </c>
       <c r="N110"/>
       <c r="P110" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B110, $C$2:$C$970, C110, $D$2:$D$970, D110, $E$2:$E$970, E110) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18786,7 +18775,7 @@
       </c>
       <c r="N111"/>
       <c r="P111" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B111, $C$2:$C$970, C111, $D$2:$D$970, D111, $E$2:$E$970, E111) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18811,7 +18800,7 @@
       </c>
       <c r="N112"/>
       <c r="P112" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B112, $C$2:$C$970, C112, $D$2:$D$970, D112, $E$2:$E$970, E112) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18836,7 +18825,7 @@
       </c>
       <c r="N113"/>
       <c r="P113" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B113, $C$2:$C$970, C113, $D$2:$D$970, D113, $E$2:$E$970, E113) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18861,7 +18850,7 @@
       </c>
       <c r="N114"/>
       <c r="P114" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B114, $C$2:$C$970, C114, $D$2:$D$970, D114, $E$2:$E$970, E114) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18886,7 +18875,7 @@
       </c>
       <c r="N115"/>
       <c r="P115" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B115, $C$2:$C$970, C115, $D$2:$D$970, D115, $E$2:$E$970, E115) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18911,7 +18900,7 @@
       </c>
       <c r="N116"/>
       <c r="P116" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B116, $C$2:$C$970, C116, $D$2:$D$970, D116, $E$2:$E$970, E116) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18936,7 +18925,7 @@
       </c>
       <c r="N117"/>
       <c r="P117" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B117, $C$2:$C$970, C117, $D$2:$D$970, D117, $E$2:$E$970, E117) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18963,7 +18952,7 @@
         <v>123</v>
       </c>
       <c r="P118" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B118, $C$2:$C$970, C118, $D$2:$D$970, D118, $E$2:$E$970, E118) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -18988,7 +18977,7 @@
       </c>
       <c r="N119"/>
       <c r="P119" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B119, $C$2:$C$970, C119, $D$2:$D$970, D119, $E$2:$E$970, E119) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19013,7 +19002,7 @@
       </c>
       <c r="N120"/>
       <c r="P120" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B120, $C$2:$C$970, C120, $D$2:$D$970, D120, $E$2:$E$970, E120) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19040,7 +19029,7 @@
         <v>125</v>
       </c>
       <c r="P121" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B121, $C$2:$C$970, C121, $D$2:$D$970, D121, $E$2:$E$970, E121) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19065,7 +19054,7 @@
       </c>
       <c r="N122"/>
       <c r="P122" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B122, $C$2:$C$970, C122, $D$2:$D$970, D122, $E$2:$E$970, E122) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19090,7 +19079,7 @@
       </c>
       <c r="N123"/>
       <c r="P123" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B123, $C$2:$C$970, C123, $D$2:$D$970, D123, $E$2:$E$970, E123) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19115,7 +19104,7 @@
       </c>
       <c r="N124"/>
       <c r="P124" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B124, $C$2:$C$970, C124, $D$2:$D$970, D124, $E$2:$E$970, E124) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19140,7 +19129,7 @@
       </c>
       <c r="N125"/>
       <c r="P125" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B125, $C$2:$C$970, C125, $D$2:$D$970, D125, $E$2:$E$970, E125) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19167,7 +19156,7 @@
         <v>123</v>
       </c>
       <c r="P126" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B126, $C$2:$C$970, C126, $D$2:$D$970, D126, $E$2:$E$970, E126) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19194,7 +19183,7 @@
         <v>123</v>
       </c>
       <c r="P127" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B127, $C$2:$C$970, C127, $D$2:$D$970, D127, $E$2:$E$970, E127) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19219,7 +19208,7 @@
       </c>
       <c r="N128"/>
       <c r="P128" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B128, $C$2:$C$970, C128, $D$2:$D$970, D128, $E$2:$E$970, E128) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19246,7 +19235,7 @@
         <v>123</v>
       </c>
       <c r="P129" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B129, $C$2:$C$970, C129, $D$2:$D$970, D129, $E$2:$E$970, E129) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="1"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19271,7 +19260,7 @@
       </c>
       <c r="N130"/>
       <c r="P130" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B130, $C$2:$C$970, C130, $D$2:$D$970, D130, $E$2:$E$970, E130) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="P130:P193" si="2">IF(COUNTIFS( $B$2:$B$970, B130, $C$2:$C$970, C130, $D$2:$D$970, D130, $E$2:$E$970, E130) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -19296,7 +19285,7 @@
       </c>
       <c r="N131"/>
       <c r="P131" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B131, $C$2:$C$970, C131, $D$2:$D$970, D131, $E$2:$E$970, E131) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19321,7 +19310,7 @@
       </c>
       <c r="N132"/>
       <c r="P132" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B132, $C$2:$C$970, C132, $D$2:$D$970, D132, $E$2:$E$970, E132) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19346,7 +19335,7 @@
       </c>
       <c r="N133"/>
       <c r="P133" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B133, $C$2:$C$970, C133, $D$2:$D$970, D133, $E$2:$E$970, E133) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19371,7 +19360,7 @@
       </c>
       <c r="N134"/>
       <c r="P134" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B134, $C$2:$C$970, C134, $D$2:$D$970, D134, $E$2:$E$970, E134) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19398,7 +19387,7 @@
         <v>123</v>
       </c>
       <c r="P135" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B135, $C$2:$C$970, C135, $D$2:$D$970, D135, $E$2:$E$970, E135) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19423,7 +19412,7 @@
       </c>
       <c r="N136"/>
       <c r="P136" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B136, $C$2:$C$970, C136, $D$2:$D$970, D136, $E$2:$E$970, E136) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19448,7 +19437,7 @@
       </c>
       <c r="N137"/>
       <c r="P137" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B137, $C$2:$C$970, C137, $D$2:$D$970, D137, $E$2:$E$970, E137) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19473,7 +19462,7 @@
       </c>
       <c r="N138"/>
       <c r="P138" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B138, $C$2:$C$970, C138, $D$2:$D$970, D138, $E$2:$E$970, E138) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19500,7 +19489,7 @@
         <v>123</v>
       </c>
       <c r="P139" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B139, $C$2:$C$970, C139, $D$2:$D$970, D139, $E$2:$E$970, E139) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19527,7 +19516,7 @@
         <v>125</v>
       </c>
       <c r="P140" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B140, $C$2:$C$970, C140, $D$2:$D$970, D140, $E$2:$E$970, E140) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19552,7 +19541,7 @@
       </c>
       <c r="N141"/>
       <c r="P141" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B141, $C$2:$C$970, C141, $D$2:$D$970, D141, $E$2:$E$970, E141) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19577,7 +19566,7 @@
       </c>
       <c r="N142"/>
       <c r="P142" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B142, $C$2:$C$970, C142, $D$2:$D$970, D142, $E$2:$E$970, E142) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19602,7 +19591,7 @@
       </c>
       <c r="N143"/>
       <c r="P143" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B143, $C$2:$C$970, C143, $D$2:$D$970, D143, $E$2:$E$970, E143) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19629,7 +19618,7 @@
         <v>125</v>
       </c>
       <c r="P144" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B144, $C$2:$C$970, C144, $D$2:$D$970, D144, $E$2:$E$970, E144) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19654,7 +19643,7 @@
       </c>
       <c r="N145"/>
       <c r="P145" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B145, $C$2:$C$970, C145, $D$2:$D$970, D145, $E$2:$E$970, E145) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19679,7 +19668,7 @@
       </c>
       <c r="N146"/>
       <c r="P146" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B146, $C$2:$C$970, C146, $D$2:$D$970, D146, $E$2:$E$970, E146) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19704,7 +19693,7 @@
       </c>
       <c r="N147"/>
       <c r="P147" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B147, $C$2:$C$970, C147, $D$2:$D$970, D147, $E$2:$E$970, E147) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19731,7 +19720,7 @@
         <v>125</v>
       </c>
       <c r="P148" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B148, $C$2:$C$970, C148, $D$2:$D$970, D148, $E$2:$E$970, E148) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19758,7 +19747,7 @@
         <v>123</v>
       </c>
       <c r="P149" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B149, $C$2:$C$970, C149, $D$2:$D$970, D149, $E$2:$E$970, E149) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19785,7 +19774,7 @@
         <v>121</v>
       </c>
       <c r="P150" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B150, $C$2:$C$970, C150, $D$2:$D$970, D150, $E$2:$E$970, E150) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19810,7 +19799,7 @@
       </c>
       <c r="N151"/>
       <c r="P151" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B151, $C$2:$C$970, C151, $D$2:$D$970, D151, $E$2:$E$970, E151) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19835,7 +19824,7 @@
       </c>
       <c r="N152"/>
       <c r="P152" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B152, $C$2:$C$970, C152, $D$2:$D$970, D152, $E$2:$E$970, E152) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19860,7 +19849,7 @@
       </c>
       <c r="N153"/>
       <c r="P153" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B153, $C$2:$C$970, C153, $D$2:$D$970, D153, $E$2:$E$970, E153) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19885,7 +19874,7 @@
       </c>
       <c r="N154"/>
       <c r="P154" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B154, $C$2:$C$970, C154, $D$2:$D$970, D154, $E$2:$E$970, E154) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19910,7 +19899,7 @@
       </c>
       <c r="N155"/>
       <c r="P155" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B155, $C$2:$C$970, C155, $D$2:$D$970, D155, $E$2:$E$970, E155) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19935,7 +19924,7 @@
       </c>
       <c r="N156"/>
       <c r="P156" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B156, $C$2:$C$970, C156, $D$2:$D$970, D156, $E$2:$E$970, E156) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19960,7 +19949,7 @@
       </c>
       <c r="N157"/>
       <c r="P157" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B157, $C$2:$C$970, C157, $D$2:$D$970, D157, $E$2:$E$970, E157) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -19985,7 +19974,7 @@
       </c>
       <c r="N158"/>
       <c r="P158" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B158, $C$2:$C$970, C158, $D$2:$D$970, D158, $E$2:$E$970, E158) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20010,7 +19999,7 @@
       </c>
       <c r="N159"/>
       <c r="P159" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B159, $C$2:$C$970, C159, $D$2:$D$970, D159, $E$2:$E$970, E159) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20037,7 +20026,7 @@
         <v>125</v>
       </c>
       <c r="P160" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B160, $C$2:$C$970, C160, $D$2:$D$970, D160, $E$2:$E$970, E160) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20062,7 +20051,7 @@
       </c>
       <c r="N161"/>
       <c r="P161" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B161, $C$2:$C$970, C161, $D$2:$D$970, D161, $E$2:$E$970, E161) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20087,7 +20076,7 @@
       </c>
       <c r="N162"/>
       <c r="P162" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B162, $C$2:$C$970, C162, $D$2:$D$970, D162, $E$2:$E$970, E162) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20112,7 +20101,7 @@
       </c>
       <c r="N163"/>
       <c r="P163" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B163, $C$2:$C$970, C163, $D$2:$D$970, D163, $E$2:$E$970, E163) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20137,7 +20126,7 @@
       </c>
       <c r="N164"/>
       <c r="P164" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B164, $C$2:$C$970, C164, $D$2:$D$970, D164, $E$2:$E$970, E164) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20162,7 +20151,7 @@
       </c>
       <c r="N165"/>
       <c r="P165" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B165, $C$2:$C$970, C165, $D$2:$D$970, D165, $E$2:$E$970, E165) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20187,7 +20176,7 @@
       </c>
       <c r="N166"/>
       <c r="P166" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B166, $C$2:$C$970, C166, $D$2:$D$970, D166, $E$2:$E$970, E166) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20212,7 +20201,7 @@
       </c>
       <c r="N167"/>
       <c r="P167" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B167, $C$2:$C$970, C167, $D$2:$D$970, D167, $E$2:$E$970, E167) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20237,7 +20226,7 @@
       </c>
       <c r="N168"/>
       <c r="P168" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B168, $C$2:$C$970, C168, $D$2:$D$970, D168, $E$2:$E$970, E168) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20262,7 +20251,7 @@
       </c>
       <c r="N169"/>
       <c r="P169" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B169, $C$2:$C$970, C169, $D$2:$D$970, D169, $E$2:$E$970, E169) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20289,7 +20278,7 @@
         <v>125</v>
       </c>
       <c r="P170" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B170, $C$2:$C$970, C170, $D$2:$D$970, D170, $E$2:$E$970, E170) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20314,7 +20303,7 @@
       </c>
       <c r="N171"/>
       <c r="P171" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B171, $C$2:$C$970, C171, $D$2:$D$970, D171, $E$2:$E$970, E171) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20341,7 +20330,7 @@
         <v>125</v>
       </c>
       <c r="P172" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B172, $C$2:$C$970, C172, $D$2:$D$970, D172, $E$2:$E$970, E172) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20366,7 +20355,7 @@
       </c>
       <c r="N173"/>
       <c r="P173" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B173, $C$2:$C$970, C173, $D$2:$D$970, D173, $E$2:$E$970, E173) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20391,7 +20380,7 @@
       </c>
       <c r="N174"/>
       <c r="P174" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B174, $C$2:$C$970, C174, $D$2:$D$970, D174, $E$2:$E$970, E174) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20416,7 +20405,7 @@
       </c>
       <c r="N175"/>
       <c r="P175" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B175, $C$2:$C$970, C175, $D$2:$D$970, D175, $E$2:$E$970, E175) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20441,7 +20430,7 @@
       </c>
       <c r="N176"/>
       <c r="P176" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B176, $C$2:$C$970, C176, $D$2:$D$970, D176, $E$2:$E$970, E176) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20466,7 +20455,7 @@
       </c>
       <c r="N177"/>
       <c r="P177" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B177, $C$2:$C$970, C177, $D$2:$D$970, D177, $E$2:$E$970, E177) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20491,7 +20480,7 @@
       </c>
       <c r="N178"/>
       <c r="P178" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B178, $C$2:$C$970, C178, $D$2:$D$970, D178, $E$2:$E$970, E178) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20516,7 +20505,7 @@
       </c>
       <c r="N179"/>
       <c r="P179" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B179, $C$2:$C$970, C179, $D$2:$D$970, D179, $E$2:$E$970, E179) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20541,7 +20530,7 @@
       </c>
       <c r="N180"/>
       <c r="P180" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B180, $C$2:$C$970, C180, $D$2:$D$970, D180, $E$2:$E$970, E180) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20566,7 +20555,7 @@
       </c>
       <c r="N181"/>
       <c r="P181" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B181, $C$2:$C$970, C181, $D$2:$D$970, D181, $E$2:$E$970, E181) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20591,7 +20580,7 @@
       </c>
       <c r="N182"/>
       <c r="P182" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B182, $C$2:$C$970, C182, $D$2:$D$970, D182, $E$2:$E$970, E182) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20616,7 +20605,7 @@
       </c>
       <c r="N183"/>
       <c r="P183" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B183, $C$2:$C$970, C183, $D$2:$D$970, D183, $E$2:$E$970, E183) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20641,7 +20630,7 @@
       </c>
       <c r="N184"/>
       <c r="P184" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B184, $C$2:$C$970, C184, $D$2:$D$970, D184, $E$2:$E$970, E184) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20666,7 +20655,7 @@
       </c>
       <c r="N185"/>
       <c r="P185" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B185, $C$2:$C$970, C185, $D$2:$D$970, D185, $E$2:$E$970, E185) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20691,7 +20680,7 @@
       </c>
       <c r="N186"/>
       <c r="P186" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B186, $C$2:$C$970, C186, $D$2:$D$970, D186, $E$2:$E$970, E186) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20716,7 +20705,7 @@
       </c>
       <c r="N187"/>
       <c r="P187" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B187, $C$2:$C$970, C187, $D$2:$D$970, D187, $E$2:$E$970, E187) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20741,7 +20730,7 @@
       </c>
       <c r="N188"/>
       <c r="P188" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B188, $C$2:$C$970, C188, $D$2:$D$970, D188, $E$2:$E$970, E188) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20766,7 +20755,7 @@
       </c>
       <c r="N189"/>
       <c r="P189" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B189, $C$2:$C$970, C189, $D$2:$D$970, D189, $E$2:$E$970, E189) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20791,7 +20780,7 @@
       </c>
       <c r="N190"/>
       <c r="P190" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B190, $C$2:$C$970, C190, $D$2:$D$970, D190, $E$2:$E$970, E190) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20818,7 +20807,7 @@
         <v>122</v>
       </c>
       <c r="P191" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B191, $C$2:$C$970, C191, $D$2:$D$970, D191, $E$2:$E$970, E191) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20843,7 +20832,7 @@
       </c>
       <c r="N192"/>
       <c r="P192" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B192, $C$2:$C$970, C192, $D$2:$D$970, D192, $E$2:$E$970, E192) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20870,7 +20859,7 @@
         <v>120</v>
       </c>
       <c r="P193" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B193, $C$2:$C$970, C193, $D$2:$D$970, D193, $E$2:$E$970, E193) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="2"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20895,7 +20884,7 @@
       </c>
       <c r="N194"/>
       <c r="P194" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B194, $C$2:$C$970, C194, $D$2:$D$970, D194, $E$2:$E$970, E194) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" ref="P194:P238" si="3">IF(COUNTIFS( $B$2:$B$970, B194, $C$2:$C$970, C194, $D$2:$D$970, D194, $E$2:$E$970, E194) &gt; 1, "Duplicate", "Unique")</f>
         <v>Unique</v>
       </c>
     </row>
@@ -20920,7 +20909,7 @@
       </c>
       <c r="N195"/>
       <c r="P195" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B195, $C$2:$C$970, C195, $D$2:$D$970, D195, $E$2:$E$970, E195) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20945,7 +20934,7 @@
       </c>
       <c r="N196"/>
       <c r="P196" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B196, $C$2:$C$970, C196, $D$2:$D$970, D196, $E$2:$E$970, E196) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20970,7 +20959,7 @@
       </c>
       <c r="N197"/>
       <c r="P197" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B197, $C$2:$C$970, C197, $D$2:$D$970, D197, $E$2:$E$970, E197) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -20995,7 +20984,7 @@
       </c>
       <c r="N198"/>
       <c r="P198" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B198, $C$2:$C$970, C198, $D$2:$D$970, D198, $E$2:$E$970, E198) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21020,7 +21009,7 @@
       </c>
       <c r="N199"/>
       <c r="P199" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B199, $C$2:$C$970, C199, $D$2:$D$970, D199, $E$2:$E$970, E199) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21047,7 +21036,7 @@
         <v>120</v>
       </c>
       <c r="P200" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B200, $C$2:$C$970, C200, $D$2:$D$970, D200, $E$2:$E$970, E200) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21072,7 +21061,7 @@
       </c>
       <c r="N201"/>
       <c r="P201" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B201, $C$2:$C$970, C201, $D$2:$D$970, D201, $E$2:$E$970, E201) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21099,7 +21088,7 @@
         <v>120</v>
       </c>
       <c r="P202" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B202, $C$2:$C$970, C202, $D$2:$D$970, D202, $E$2:$E$970, E202) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21124,7 +21113,7 @@
       </c>
       <c r="N203"/>
       <c r="P203" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B203, $C$2:$C$970, C203, $D$2:$D$970, D203, $E$2:$E$970, E203) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21149,7 +21138,7 @@
       </c>
       <c r="N204"/>
       <c r="P204" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B204, $C$2:$C$970, C204, $D$2:$D$970, D204, $E$2:$E$970, E204) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21176,7 +21165,7 @@
         <v>124</v>
       </c>
       <c r="P205" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B205, $C$2:$C$970, C205, $D$2:$D$970, D205, $E$2:$E$970, E205) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21201,7 +21190,7 @@
       </c>
       <c r="N206"/>
       <c r="P206" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B206, $C$2:$C$970, C206, $D$2:$D$970, D206, $E$2:$E$970, E206) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21226,7 +21215,7 @@
       </c>
       <c r="N207"/>
       <c r="P207" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B207, $C$2:$C$970, C207, $D$2:$D$970, D207, $E$2:$E$970, E207) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21251,7 +21240,7 @@
       </c>
       <c r="N208"/>
       <c r="P208" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B208, $C$2:$C$970, C208, $D$2:$D$970, D208, $E$2:$E$970, E208) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21276,7 +21265,7 @@
       </c>
       <c r="N209"/>
       <c r="P209" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B209, $C$2:$C$970, C209, $D$2:$D$970, D209, $E$2:$E$970, E209) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21301,7 +21290,7 @@
       </c>
       <c r="N210"/>
       <c r="P210" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B210, $C$2:$C$970, C210, $D$2:$D$970, D210, $E$2:$E$970, E210) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21328,7 +21317,7 @@
         <v>124</v>
       </c>
       <c r="P211" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B211, $C$2:$C$970, C211, $D$2:$D$970, D211, $E$2:$E$970, E211) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21353,7 +21342,7 @@
       </c>
       <c r="N212"/>
       <c r="P212" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B212, $C$2:$C$970, C212, $D$2:$D$970, D212, $E$2:$E$970, E212) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21378,7 +21367,7 @@
       </c>
       <c r="N213"/>
       <c r="P213" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B213, $C$2:$C$970, C213, $D$2:$D$970, D213, $E$2:$E$970, E213) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21403,7 +21392,7 @@
       </c>
       <c r="N214"/>
       <c r="P214" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B214, $C$2:$C$970, C214, $D$2:$D$970, D214, $E$2:$E$970, E214) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21428,7 +21417,7 @@
       </c>
       <c r="N215"/>
       <c r="P215" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B215, $C$2:$C$970, C215, $D$2:$D$970, D215, $E$2:$E$970, E215) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21453,7 +21442,7 @@
       </c>
       <c r="N216"/>
       <c r="P216" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B216, $C$2:$C$970, C216, $D$2:$D$970, D216, $E$2:$E$970, E216) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21478,7 +21467,7 @@
       </c>
       <c r="N217"/>
       <c r="P217" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B217, $C$2:$C$970, C217, $D$2:$D$970, D217, $E$2:$E$970, E217) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21503,7 +21492,7 @@
       </c>
       <c r="N218"/>
       <c r="P218" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B218, $C$2:$C$970, C218, $D$2:$D$970, D218, $E$2:$E$970, E218) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21528,7 +21517,7 @@
       </c>
       <c r="N219"/>
       <c r="P219" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B219, $C$2:$C$970, C219, $D$2:$D$970, D219, $E$2:$E$970, E219) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21555,7 +21544,7 @@
         <v>120</v>
       </c>
       <c r="P220" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B220, $C$2:$C$970, C220, $D$2:$D$970, D220, $E$2:$E$970, E220) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21580,7 +21569,7 @@
       </c>
       <c r="N221"/>
       <c r="P221" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B221, $C$2:$C$970, C221, $D$2:$D$970, D221, $E$2:$E$970, E221) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21605,7 +21594,7 @@
       </c>
       <c r="N222"/>
       <c r="P222" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B222, $C$2:$C$970, C222, $D$2:$D$970, D222, $E$2:$E$970, E222) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21630,7 +21619,7 @@
       </c>
       <c r="N223"/>
       <c r="P223" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B223, $C$2:$C$970, C223, $D$2:$D$970, D223, $E$2:$E$970, E223) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21655,7 +21644,7 @@
       </c>
       <c r="N224"/>
       <c r="P224" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B224, $C$2:$C$970, C224, $D$2:$D$970, D224, $E$2:$E$970, E224) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21680,7 +21669,7 @@
       </c>
       <c r="N225"/>
       <c r="P225" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B225, $C$2:$C$970, C225, $D$2:$D$970, D225, $E$2:$E$970, E225) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21705,7 +21694,7 @@
       </c>
       <c r="N226"/>
       <c r="P226" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B226, $C$2:$C$970, C226, $D$2:$D$970, D226, $E$2:$E$970, E226) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21730,7 +21719,7 @@
       </c>
       <c r="N227"/>
       <c r="P227" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B227, $C$2:$C$970, C227, $D$2:$D$970, D227, $E$2:$E$970, E227) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21755,7 +21744,7 @@
       </c>
       <c r="N228"/>
       <c r="P228" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B228, $C$2:$C$970, C228, $D$2:$D$970, D228, $E$2:$E$970, E228) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21780,7 +21769,7 @@
       </c>
       <c r="N229"/>
       <c r="P229" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B229, $C$2:$C$970, C229, $D$2:$D$970, D229, $E$2:$E$970, E229) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21805,7 +21794,7 @@
       </c>
       <c r="N230"/>
       <c r="P230" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B230, $C$2:$C$970, C230, $D$2:$D$970, D230, $E$2:$E$970, E230) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21830,7 +21819,7 @@
       </c>
       <c r="N231"/>
       <c r="P231" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B231, $C$2:$C$970, C231, $D$2:$D$970, D231, $E$2:$E$970, E231) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21855,7 +21844,7 @@
       </c>
       <c r="N232"/>
       <c r="P232" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B232, $C$2:$C$970, C232, $D$2:$D$970, D232, $E$2:$E$970, E232) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21882,7 +21871,7 @@
         <v>120</v>
       </c>
       <c r="P233" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B233, $C$2:$C$970, C233, $D$2:$D$970, D233, $E$2:$E$970, E233) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21910,7 +21899,7 @@
         <v>120</v>
       </c>
       <c r="P234" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B234, $C$2:$C$970, C234, $D$2:$D$970, D234, $E$2:$E$970, E234) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21937,7 +21926,7 @@
         <v>120</v>
       </c>
       <c r="P235" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B235, $C$2:$C$970, C235, $D$2:$D$970, D235, $E$2:$E$970, E235) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21962,7 +21951,7 @@
       </c>
       <c r="N236"/>
       <c r="P236" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B236, $C$2:$C$970, C236, $D$2:$D$970, D236, $E$2:$E$970, E236) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -21989,7 +21978,7 @@
         <v>117</v>
       </c>
       <c r="P237" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B237, $C$2:$C$970, C237, $D$2:$D$970, D237, $E$2:$E$970, E237) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>
@@ -22016,7 +22005,7 @@
         <v>120</v>
       </c>
       <c r="P238" s="22" t="str">
-        <f>IF(COUNTIFS( $B$2:$B$970, B238, $C$2:$C$970, C238, $D$2:$D$970, D238, $E$2:$E$970, E238) &gt; 1, "Duplicate", "Unique")</f>
+        <f t="shared" si="3"/>
         <v>Unique</v>
       </c>
     </row>

</xml_diff>